<commit_message>
add squareroot and power
</commit_message>
<xml_diff>
--- a/TESTE E REPORT - CALCULADORA.xlsx
+++ b/TESTE E REPORT - CALCULADORA.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="150">
   <si>
     <t>Resumo</t>
   </si>
@@ -161,46 +161,43 @@
     <t>Calculadora</t>
   </si>
   <si>
-    <t>Soma</t>
-  </si>
-  <si>
-    <t>Chamar a função somar, e enviar como primeiro parametro 1, como segundo parametro 99</t>
-  </si>
-  <si>
-    <t>A função irá retornar 100</t>
-  </si>
-  <si>
-    <t>Chamar a função somar, e enviar como primeiro parametro -1, como segundo parametro 99</t>
-  </si>
-  <si>
-    <t>A função irá retornar 98</t>
-  </si>
-  <si>
-    <t>Chamar a função somar, e enviar como primeiro parametro 1, como segundo parametro -99</t>
-  </si>
-  <si>
-    <t>A função irá retornar -98</t>
-  </si>
-  <si>
-    <t>Chamar a função somar, e enviar como primeiro parametro -1, como segundo parametro -99</t>
-  </si>
-  <si>
-    <t>A função irá retornar -100</t>
-  </si>
-  <si>
-    <t>Chamar a função somar, e enviar como primeiro parametro 1.5, como segundo parametro 2.3</t>
-  </si>
-  <si>
-    <t>A função irá retornar 3.8</t>
-  </si>
-  <si>
-    <t>Chamar a função somar, e enviar como primeiro parametro 'batata', como segundo parametro 1</t>
+    <t>Adição</t>
+  </si>
+  <si>
+    <t>Chamar a função somar, e enviar como primeiro parametro 2, como segundo parametro 95</t>
+  </si>
+  <si>
+    <t>A função irá retornar 97</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Chamar a função somar, e enviar como primeiro parametro -5, como segundo parametro 10</t>
+  </si>
+  <si>
+    <t>A função irá retornar 5</t>
+  </si>
+  <si>
+    <t>Chamar a função somar, e enviar como primeiro parametro 10, como segundo parametro -5</t>
+  </si>
+  <si>
+    <t>Chamar a função somar, e enviar como primeiro parametro -5, como segundo parametro -10</t>
+  </si>
+  <si>
+    <t>A função irá retornar -15</t>
+  </si>
+  <si>
+    <t>Chamar a função somar, e enviar como primeiro parametro 0.5, como segundo parametro 1.7</t>
+  </si>
+  <si>
+    <t>A função irá retornar 2.2</t>
+  </si>
+  <si>
+    <t>Chamar a função somar, e enviar como primeiro parametro 'a', como segundo parametro 1</t>
   </si>
   <si>
     <t>A função irá retornar um erro - Enviar somente números</t>
   </si>
   <si>
-    <t>Chamar a função somar, e enviar como primeiro parametro 1, como segundo parametro 'batata'</t>
+    <t>Chamar a função somar, e enviar como primeiro parametro 1, como segundo parametro 'a'</t>
   </si>
   <si>
     <t>Chamar a função somar, e enviar como primeiro parametro 0, como segundo parametro 1</t>
@@ -212,152 +209,269 @@
     <t>Chamar a função somar, e enviar como primeiro parametro 1, como segundo parametro 0</t>
   </si>
   <si>
+    <t xml:space="preserve">Chamar a função somar sem o primeiro parâmetro </t>
+  </si>
+  <si>
+    <t xml:space="preserve">A função irá retornar um erro - Envie todos os campos!           </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chamar a função somar sem o segundo parâmetro </t>
+  </si>
+  <si>
+    <t>A função irá retornar um erro - Envie todos os campos!</t>
+  </si>
+  <si>
+    <t>Chamar a função somar sem os dois parâmetros</t>
+  </si>
+  <si>
     <t>Subtração</t>
   </si>
   <si>
-    <t>Chamar a função subtrair, e enviar como primeiro parametro 2, como segundo parametro 1</t>
-  </si>
-  <si>
-    <t>Chamar a função subtrair, e enviar como primeiro parametro 1, como segundo parametro 2</t>
+    <t>Chamar a função subtrair, e enviar como primeiro parametro 2, como segundo parametro 95</t>
+  </si>
+  <si>
+    <t>A função irá retornar -93</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Chamar a função subtrair, e enviar como primeiro parametro -5, como segundo parametro 10</t>
+  </si>
+  <si>
+    <t>Chamar a função subtrair, e enviar como primeiro parametro 10, como segundo parametro -5</t>
+  </si>
+  <si>
+    <t>A função irá retornar 15</t>
+  </si>
+  <si>
+    <t>Chamar a função subtrair, e enviar como primeiro parametro -5, como segundo parametro -10</t>
+  </si>
+  <si>
+    <t>Chamar a função subtrair, e enviar como primeiro parametro 0.5, como segundo parametro 1.7</t>
+  </si>
+  <si>
+    <t>A função irá retornar -1.2</t>
+  </si>
+  <si>
+    <t>Chamar a função subtrair, e enviar como primeiro parametro 'a', como segundo parametro 1</t>
+  </si>
+  <si>
+    <t>Chamar a função subtrair, e enviar como primeiro parametro 1, como segundo parametro 'a'</t>
+  </si>
+  <si>
+    <t>Chamar a função subtrair, e enviar como primeiro parametro 0, como segundo parametro 1</t>
   </si>
   <si>
     <t>A função irá retornar -1</t>
   </si>
   <si>
-    <t>Chamar a função subtrair, e enviar como primeiro parametro -1, como segundo parametro 2</t>
-  </si>
-  <si>
-    <t>A função irá retornar -3</t>
-  </si>
-  <si>
-    <t>Chamar a função subtrair, e enviar como primeiro parametro 1, como segundo parametro -2</t>
-  </si>
-  <si>
-    <t>A função irá retornar 3</t>
-  </si>
-  <si>
-    <t>Chamar a função subtrair, e enviar como primeiro parametro 0, como segundo parametro 2</t>
+    <t>Chamar a função subtrair, e enviar como primeiro parametro 1, como segundo parametro 0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chamar a função subtrair sem o primeiro parâmetro </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chamar a função subtrair sem o segundo parâmetro </t>
+  </si>
+  <si>
+    <t>Chamar a função subtrair sem os dois parâmetros</t>
+  </si>
+  <si>
+    <t>Mutiplicação</t>
+  </si>
+  <si>
+    <t>Chamar a função multiplicar, e enviar como primeiro parametro 2, como segundo parametro 95</t>
+  </si>
+  <si>
+    <t>A função irá retornar 190</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Chamar a função multiplicar, e enviar como primeiro parametro -5, como segundo parametro 10</t>
+  </si>
+  <si>
+    <t>A função irá retornar -50</t>
+  </si>
+  <si>
+    <t>Chamar a função multiplicar, e enviar como primeiro parametro 10, como segundo parametro -5</t>
+  </si>
+  <si>
+    <t>Chamar a função multiplicar, e enviar como primeiro parametro -5, como segundo parametro -10</t>
+  </si>
+  <si>
+    <t>A função irá retornar 50</t>
+  </si>
+  <si>
+    <t>Chamar a função multiplicar, e enviar como primeiro parametro 0.5, como segundo parametro 1.7</t>
+  </si>
+  <si>
+    <t>A função irá retornar 0.85</t>
+  </si>
+  <si>
+    <t>Chamar a função multiplicar, e enviar como primeiro parametro 'a', como segundo parametro 1</t>
+  </si>
+  <si>
+    <t>Chamar a função multiplicar, e enviar como primeiro parametro 1, como segundo parametro 'a'</t>
+  </si>
+  <si>
+    <t>Chamar a função multiplicar, e enviar como primeiro parametro 0, como segundo parametro 1</t>
+  </si>
+  <si>
+    <t>A função irá retornar 0</t>
+  </si>
+  <si>
+    <t>Chamar a função multiplicar, e enviar como primeiro parametro 1, como segundo parametro 0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chamar a função multiplicar sem o primeiro parâmetro </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chamar a função multiplicar sem o segundo parâmetro </t>
+  </si>
+  <si>
+    <t>Chamar a função multiplicar sem os dois parâmetros</t>
+  </si>
+  <si>
+    <t>Divisão</t>
+  </si>
+  <si>
+    <t>Chamar a função dividir, e enviar como primeiro parametro 2, como segundo parametro 95</t>
+  </si>
+  <si>
+    <t>A função irá retornar 0.02105263157</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Chamar a função dividir, e enviar como primeiro parametro -5, como segundo parametro 10</t>
+  </si>
+  <si>
+    <t>A função irá retornar -0.5</t>
+  </si>
+  <si>
+    <t>Chamar a função dividir, e enviar como primeiro parametro 10, como segundo parametro -5</t>
   </si>
   <si>
     <t>A função irá retornar -2</t>
   </si>
   <si>
-    <t>Chamar a função subtrair, e enviar como primeiro parametro 2, como segundo parametro 0</t>
-  </si>
-  <si>
-    <t>A função irá retornar 0</t>
-  </si>
-  <si>
-    <t>Chamar a função subtrair, e enviar como primeiro parametro 'a', como segundo parametro 1</t>
-  </si>
-  <si>
-    <t>Chamar a função subtrair, e enviar como primeiro parametro 2, como segundo parametro 'a'</t>
-  </si>
-  <si>
-    <t>Chamar a função subtrair, e enviar como primeiro parametro 3.5, como segundo parametro 1.7</t>
-  </si>
-  <si>
-    <t>A função irá retornar 1.8</t>
-  </si>
-  <si>
-    <t>Multiplicação</t>
-  </si>
-  <si>
-    <t>Chamar a função multiplicar, e enviar como primeiro parametro 3, como segundo parametro 2</t>
-  </si>
-  <si>
-    <t>A função irá retornar 6</t>
-  </si>
-  <si>
-    <t>Chamar a função multiplicar, e enviar como primeiro parametro -3, como segundo parametro 2</t>
-  </si>
-  <si>
-    <t>A função irá retornar -6</t>
-  </si>
-  <si>
-    <t>Chamar a função multiplicar, e enviar como primeiro parametro 3, como segundo parametro -4</t>
-  </si>
-  <si>
-    <t>A função irá retornar -8</t>
-  </si>
-  <si>
-    <t>Chamar a função multiplicar, e enviar como primeiro parametro 2.3, como segundo parametro 1.8</t>
-  </si>
-  <si>
-    <t>A função irá retornar 4.14</t>
-  </si>
-  <si>
-    <t>Chamar a função multiplicar, e enviar como primeiro parametro 3, como segundo parametro 0</t>
-  </si>
-  <si>
-    <t>Chamar a função multiplicar, e enviar como primeiro parametro 0, como segundo parametro 3</t>
-  </si>
-  <si>
-    <t>Chamar a função multiplicar, e enviar como primeiro parametro 'b', como segundo parametro 3</t>
-  </si>
-  <si>
-    <t>Chamar a função multiplicar, e enviar como primeiro parametro 3, como segundo parametro 'b"</t>
-  </si>
-  <si>
-    <t>Chamar a função multiplicar, e enviar como primeiro parametro  -3, como segundo parametro  -4</t>
-  </si>
-  <si>
-    <t>A função irá retornar 12</t>
-  </si>
-  <si>
-    <t>Divisão</t>
-  </si>
-  <si>
-    <t>Chamar a função dividir, e enviar como primeiro parametro  12, como segundo parametro  2</t>
-  </si>
-  <si>
-    <t>Chamar a função dividir, e enviar como primeiro parametro  2, como segundo parametro  4</t>
-  </si>
-  <si>
-    <t>A função irá retornar 0.5</t>
-  </si>
-  <si>
-    <t>Chamar a função dividir, e enviar como primeiro parametro  12, como segundo parametro  0.5</t>
-  </si>
-  <si>
-    <t>A função irá retornar 24</t>
-  </si>
-  <si>
-    <t>Chamar a função dividir, e enviar como primeiro parametro  0.8, como segundo parametro  2</t>
-  </si>
-  <si>
-    <t>A função irá retornar 0.4</t>
-  </si>
-  <si>
-    <t>Chamar a função dividir, e enviar como primeiro parametro  0, como segundo parametro  2</t>
-  </si>
-  <si>
-    <t>Chamar a função dividir, e enviar como primeiro parametro  2, como segundo parametro  0</t>
-  </si>
-  <si>
-    <t>A função irá retornar um erro - Não é possível dividir por zero</t>
-  </si>
-  <si>
-    <t>Chamar a função dividir, e enviar como primeiro parametro  'a', como segundo parametro 2</t>
-  </si>
-  <si>
-    <t>Chamar a função dividir, e enviar como primeiro parametro  -6, como segundo parametro -3</t>
+    <t>Chamar a função dividir, e enviar como primeiro parametro -5, como segundo parametro -10</t>
+  </si>
+  <si>
+    <t>Chamar a função dividir, e enviar como primeiro parametro 0.5, como segundo parametro 1.7</t>
+  </si>
+  <si>
+    <t>A função irá retornar 0.2941176</t>
+  </si>
+  <si>
+    <t>Chamar a função dividir, e enviar como primeiro parametro 'a', como segundo parametro 1</t>
+  </si>
+  <si>
+    <t>Chamar a função dividir, e enviar como primeiro parametro 1, como segundo parametro 'a'</t>
+  </si>
+  <si>
+    <t>Chamar a função dividir, e enviar como primeiro parametro 0, como segundo parametro 1</t>
+  </si>
+  <si>
+    <t>Chamar a função dividir, e enviar como primeiro parametro 1, como segundo parametro 0</t>
+  </si>
+  <si>
+    <t>A função irá retornar Undefined</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chamar a função dividir sem o primeiro parâmetro </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chamar a função dividir sem o segundo parâmetro </t>
+  </si>
+  <si>
+    <t>Chamar a função dividir sem os dois parâmetros</t>
+  </si>
+  <si>
+    <t>Potencia</t>
+  </si>
+  <si>
+    <t>Chamar a função potencia, e enviar como primeiro parametro 2, como segundo parametro 5</t>
+  </si>
+  <si>
+    <t>A função irá retornar 32</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Chamar a função potencia, e enviar como primeiro parametro -5, como segundo parametro 5</t>
+  </si>
+  <si>
+    <t>A função irá retornar -3125</t>
+  </si>
+  <si>
+    <t>Chamar a função potencia, e enviar como primeiro parametro 10, como segundo parametro -2</t>
+  </si>
+  <si>
+    <t>A função irá retornar 0.01</t>
+  </si>
+  <si>
+    <t>Chamar a função potencia, e enviar como primeiro parametro -5, como segundo parametro -2</t>
+  </si>
+  <si>
+    <t>A função irá retornar 0.04</t>
+  </si>
+  <si>
+    <t>Chamar a função potencia, e enviar como primeiro parametro 0.5, como segundo parametro 2</t>
+  </si>
+  <si>
+    <t>A função irá retornar 0.25</t>
+  </si>
+  <si>
+    <t>Chamar a função potencia, e enviar como primeiro parametro 'a', como segundo parametro 1</t>
+  </si>
+  <si>
+    <t>Chamar a função potencia, e enviar como primeiro parametro 1, como segundo parametro 'a'</t>
+  </si>
+  <si>
+    <t>Chamar a função potencia, e enviar como primeiro parametro 0, como segundo parametro 1</t>
+  </si>
+  <si>
+    <t>Chamar a função potencia, e enviar como primeiro parametro 1, como segundo parametro 0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chamar a função potencia sem o primeiro parâmetro </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chamar a função potencia sem o segundo parâmetro </t>
+  </si>
+  <si>
+    <t>Chamar a função potencia sem os dois parâmetros</t>
+  </si>
+  <si>
+    <t>Raiz</t>
+  </si>
+  <si>
+    <t>Chamar a função raiz, e enviar como parametro 4</t>
   </si>
   <si>
     <t>A função irá retornar 2</t>
   </si>
   <si>
-    <t>Data: 27/03/2026</t>
-  </si>
-  <si>
-    <t>Autor: Pablo Ricardo Paul</t>
+    <t>Chamar a função raiz, e enviar como parametro -9</t>
+  </si>
+  <si>
+    <t>A função irá retornar erro - Não é possível calcular a raiz de um número negativo</t>
+  </si>
+  <si>
+    <t>Chamar a função raiz, e enviar como parametro 1.8</t>
+  </si>
+  <si>
+    <t>A função irá retornar 1.3416407864998738</t>
+  </si>
+  <si>
+    <t>Chamar a função raiz, e enviar como parametro 'a'</t>
+  </si>
+  <si>
+    <t>Chamar a função raiz, e enviar como parametro 0</t>
+  </si>
+  <si>
+    <t>Chamar a função raiz sem o parâmetro</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="14">
+  <fonts count="13">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -419,11 +533,6 @@
       <name val="Arial"/>
     </font>
     <font/>
-    <font>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
   <fills count="7">
     <fill>
@@ -513,7 +622,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="39">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -608,15 +717,24 @@
       <alignment horizontal="center" vertical="bottom"/>
     </xf>
     <xf borderId="2" fillId="3" fontId="3" numFmtId="4" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="3" fontId="3" numFmtId="3" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="3" fillId="0" fontId="12" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="4" fillId="0" fontId="12" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="0" fillId="3" fontId="3" numFmtId="4" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf borderId="2" fillId="3" fontId="3" numFmtId="4" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="3" fillId="0" fontId="12" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="4" fillId="0" fontId="12" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1842,10 +1960,10 @@
       <c r="A6" s="31" t="s">
         <v>47</v>
       </c>
-      <c r="B6" s="32" t="s">
+      <c r="B6" s="31" t="s">
         <v>48</v>
       </c>
-      <c r="C6" s="23">
+      <c r="C6" s="32">
         <v>1.0</v>
       </c>
       <c r="D6" s="27" t="s">
@@ -1854,597 +1972,1062 @@
       <c r="E6" s="27" t="s">
         <v>50</v>
       </c>
-      <c r="F6" s="25" t="b">
+      <c r="F6" s="33" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="33"/>
-      <c r="B7" s="33"/>
-      <c r="C7" s="23">
+      <c r="A7" s="34"/>
+      <c r="B7" s="34"/>
+      <c r="C7" s="32">
         <v>2.0</v>
       </c>
-      <c r="D7" s="26" t="s">
+      <c r="D7" s="27" t="s">
         <v>51</v>
       </c>
       <c r="E7" s="27" t="s">
         <v>52</v>
       </c>
-      <c r="F7" s="25" t="b">
+      <c r="F7" s="33" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="33"/>
-      <c r="B8" s="33"/>
-      <c r="C8" s="23">
+      <c r="A8" s="34"/>
+      <c r="B8" s="34"/>
+      <c r="C8" s="32">
         <v>3.0</v>
       </c>
       <c r="D8" s="27" t="s">
         <v>53</v>
       </c>
       <c r="E8" s="27" t="s">
+        <v>52</v>
+      </c>
+      <c r="F8" s="33" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="34"/>
+      <c r="B9" s="34"/>
+      <c r="C9" s="32">
+        <v>4.0</v>
+      </c>
+      <c r="D9" s="27" t="s">
         <v>54</v>
       </c>
-      <c r="F8" s="25" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="33"/>
-      <c r="B9" s="33"/>
-      <c r="C9" s="23">
-        <v>4.0</v>
-      </c>
-      <c r="D9" s="27" t="s">
+      <c r="E9" s="27" t="s">
         <v>55</v>
       </c>
-      <c r="E9" s="27" t="s">
+      <c r="F9" s="33" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="34"/>
+      <c r="B10" s="34"/>
+      <c r="C10" s="32">
+        <v>5.0</v>
+      </c>
+      <c r="D10" s="27" t="s">
         <v>56</v>
       </c>
-      <c r="F9" s="25" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="33"/>
-      <c r="B10" s="33"/>
-      <c r="C10" s="23">
-        <v>5.0</v>
-      </c>
-      <c r="D10" s="27" t="s">
+      <c r="E10" s="27" t="s">
         <v>57</v>
       </c>
-      <c r="E10" s="27" t="s">
+      <c r="F10" s="33" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="34"/>
+      <c r="B11" s="34"/>
+      <c r="C11" s="32">
+        <v>6.0</v>
+      </c>
+      <c r="D11" s="27" t="s">
         <v>58</v>
       </c>
-      <c r="F10" s="25" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="33"/>
-      <c r="B11" s="33"/>
-      <c r="C11" s="23">
-        <v>6.0</v>
-      </c>
-      <c r="D11" s="27" t="s">
+      <c r="E11" s="27" t="s">
         <v>59</v>
       </c>
-      <c r="E11" s="27" t="s">
+      <c r="F11" s="33" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="34"/>
+      <c r="B12" s="34"/>
+      <c r="C12" s="32">
+        <v>7.0</v>
+      </c>
+      <c r="D12" s="27" t="s">
         <v>60</v>
       </c>
-      <c r="F11" s="25" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="33"/>
-      <c r="B12" s="33"/>
-      <c r="C12" s="23">
-        <v>7.0</v>
-      </c>
-      <c r="D12" s="27" t="s">
+      <c r="E12" s="27" t="s">
+        <v>59</v>
+      </c>
+      <c r="F12" s="33" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="34"/>
+      <c r="B13" s="34"/>
+      <c r="C13" s="32">
+        <v>8.0</v>
+      </c>
+      <c r="D13" s="27" t="s">
         <v>61</v>
       </c>
-      <c r="E12" s="27" t="s">
-        <v>60</v>
-      </c>
-      <c r="F12" s="25" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="33"/>
-      <c r="B13" s="33"/>
-      <c r="C13" s="23">
-        <v>8.0</v>
-      </c>
-      <c r="D13" s="27" t="s">
+      <c r="E13" s="27" t="s">
         <v>62</v>
       </c>
-      <c r="E13" s="27" t="s">
+      <c r="F13" s="33" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="34"/>
+      <c r="B14" s="34"/>
+      <c r="C14" s="32">
+        <v>9.0</v>
+      </c>
+      <c r="D14" s="27" t="s">
         <v>63</v>
       </c>
-      <c r="F13" s="25" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="33"/>
-      <c r="B14" s="34"/>
-      <c r="C14" s="23">
-        <v>9.0</v>
-      </c>
-      <c r="D14" s="27" t="s">
+      <c r="E14" s="27" t="s">
+        <v>62</v>
+      </c>
+      <c r="F14" s="33" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="34"/>
+      <c r="B15" s="34"/>
+      <c r="C15" s="32">
+        <v>10.0</v>
+      </c>
+      <c r="D15" s="27" t="s">
         <v>64</v>
       </c>
-      <c r="E14" s="27" t="s">
-        <v>63</v>
-      </c>
-      <c r="F14" s="25" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="33"/>
-      <c r="B15" s="32" t="s">
+      <c r="E15" s="27" t="s">
         <v>65</v>
       </c>
-      <c r="C15" s="23">
-        <v>10.0</v>
-      </c>
-      <c r="D15" s="24" t="s">
+      <c r="F15" s="33" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="34"/>
+      <c r="B16" s="34"/>
+      <c r="C16" s="32">
+        <v>11.0</v>
+      </c>
+      <c r="D16" s="27" t="s">
         <v>66</v>
       </c>
-      <c r="E15" s="24" t="s">
-        <v>63</v>
-      </c>
-      <c r="F15" s="25" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="33"/>
-      <c r="B16" s="33"/>
-      <c r="C16" s="23">
-        <v>11.0</v>
-      </c>
-      <c r="D16" s="24" t="s">
+      <c r="E16" s="27" t="s">
         <v>67</v>
       </c>
-      <c r="E16" s="24" t="s">
+      <c r="F16" s="33" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="34"/>
+      <c r="B17" s="34"/>
+      <c r="C17" s="32">
+        <v>12.0</v>
+      </c>
+      <c r="D17" s="27" t="s">
         <v>68</v>
       </c>
-      <c r="F16" s="25" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="33"/>
-      <c r="B17" s="33"/>
-      <c r="C17" s="23">
-        <v>12.0</v>
-      </c>
-      <c r="D17" s="24" t="s">
+      <c r="E17" s="27" t="s">
+        <v>67</v>
+      </c>
+      <c r="F17" s="33" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="34"/>
+      <c r="B18" s="31" t="s">
         <v>69</v>
       </c>
-      <c r="E17" s="24" t="s">
+      <c r="C18" s="32">
+        <v>13.0</v>
+      </c>
+      <c r="D18" s="27" t="s">
         <v>70</v>
       </c>
-      <c r="F17" s="25" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="33"/>
-      <c r="B18" s="33"/>
-      <c r="C18" s="23">
-        <v>13.0</v>
-      </c>
-      <c r="D18" s="24" t="s">
+      <c r="E18" s="27" t="s">
         <v>71</v>
       </c>
-      <c r="E18" s="24" t="s">
+      <c r="F18" s="33" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="34"/>
+      <c r="B19" s="34"/>
+      <c r="C19" s="32">
+        <v>14.0</v>
+      </c>
+      <c r="D19" s="27" t="s">
         <v>72</v>
       </c>
-      <c r="F18" s="25" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="33"/>
-      <c r="B19" s="33"/>
-      <c r="C19" s="23">
-        <v>14.0</v>
-      </c>
-      <c r="D19" s="24" t="s">
+      <c r="E19" s="27" t="s">
+        <v>55</v>
+      </c>
+      <c r="F19" s="33" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="34"/>
+      <c r="B20" s="34"/>
+      <c r="C20" s="32">
+        <v>15.0</v>
+      </c>
+      <c r="D20" s="27" t="s">
         <v>73</v>
       </c>
-      <c r="E19" s="24" t="s">
+      <c r="E20" s="27" t="s">
         <v>74</v>
       </c>
-      <c r="F19" s="25" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="33"/>
-      <c r="B20" s="33"/>
-      <c r="C20" s="23">
-        <v>15.0</v>
-      </c>
-      <c r="D20" s="24" t="s">
+      <c r="F20" s="33" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="34"/>
+      <c r="B21" s="34"/>
+      <c r="C21" s="32">
+        <v>16.0</v>
+      </c>
+      <c r="D21" s="27" t="s">
         <v>75</v>
       </c>
-      <c r="E20" s="24" t="s">
+      <c r="E21" s="27" t="s">
+        <v>52</v>
+      </c>
+      <c r="F21" s="33" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="34"/>
+      <c r="B22" s="34"/>
+      <c r="C22" s="32">
+        <v>17.0</v>
+      </c>
+      <c r="D22" s="27" t="s">
         <v>76</v>
       </c>
-      <c r="F20" s="25" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="33"/>
-      <c r="B21" s="33"/>
-      <c r="C21" s="23">
-        <v>16.0</v>
-      </c>
-      <c r="D21" s="24" t="s">
+      <c r="E22" s="27" t="s">
         <v>77</v>
       </c>
-      <c r="E21" s="24" t="s">
-        <v>60</v>
-      </c>
-      <c r="F21" s="25" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="33"/>
-      <c r="B22" s="33"/>
-      <c r="C22" s="23">
-        <v>17.0</v>
-      </c>
-      <c r="D22" s="24" t="s">
+      <c r="F22" s="33" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="34"/>
+      <c r="B23" s="34"/>
+      <c r="C23" s="32">
+        <v>18.0</v>
+      </c>
+      <c r="D23" s="27" t="s">
         <v>78</v>
       </c>
-      <c r="E22" s="24" t="s">
-        <v>60</v>
-      </c>
-      <c r="F22" s="25" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="33"/>
-      <c r="B23" s="34"/>
-      <c r="C23" s="23">
-        <v>18.0</v>
-      </c>
-      <c r="D23" s="24" t="s">
+      <c r="E23" s="27" t="s">
+        <v>59</v>
+      </c>
+      <c r="F23" s="33" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="34"/>
+      <c r="B24" s="34"/>
+      <c r="C24" s="32">
+        <v>19.0</v>
+      </c>
+      <c r="D24" s="27" t="s">
         <v>79</v>
       </c>
-      <c r="E23" s="24" t="s">
+      <c r="E24" s="27" t="s">
+        <v>59</v>
+      </c>
+      <c r="F24" s="33" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="34"/>
+      <c r="B25" s="34"/>
+      <c r="C25" s="32">
+        <v>20.0</v>
+      </c>
+      <c r="D25" s="27" t="s">
         <v>80</v>
       </c>
-      <c r="F23" s="25" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="33"/>
-      <c r="B24" s="32" t="s">
+      <c r="E25" s="27" t="s">
         <v>81</v>
       </c>
-      <c r="C24" s="23">
-        <v>19.0</v>
-      </c>
-      <c r="D24" s="24" t="s">
+      <c r="F25" s="33" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="34"/>
+      <c r="B26" s="34"/>
+      <c r="C26" s="32">
+        <v>21.0</v>
+      </c>
+      <c r="D26" s="27" t="s">
         <v>82</v>
       </c>
-      <c r="E24" s="24" t="s">
+      <c r="E26" s="27" t="s">
+        <v>62</v>
+      </c>
+      <c r="F26" s="33" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="34"/>
+      <c r="B27" s="34"/>
+      <c r="C27" s="32">
+        <v>22.0</v>
+      </c>
+      <c r="D27" s="27" t="s">
         <v>83</v>
       </c>
-      <c r="F24" s="25" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="33"/>
-      <c r="B25" s="33"/>
-      <c r="C25" s="23">
-        <v>20.0</v>
-      </c>
-      <c r="D25" s="24" t="s">
+      <c r="E27" s="27" t="s">
+        <v>65</v>
+      </c>
+      <c r="F27" s="33" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="34"/>
+      <c r="B28" s="34"/>
+      <c r="C28" s="32">
+        <v>23.0</v>
+      </c>
+      <c r="D28" s="27" t="s">
         <v>84</v>
       </c>
-      <c r="E25" s="24" t="s">
+      <c r="E28" s="27" t="s">
+        <v>65</v>
+      </c>
+      <c r="F28" s="33" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="34"/>
+      <c r="B29" s="35"/>
+      <c r="C29" s="32">
+        <v>24.0</v>
+      </c>
+      <c r="D29" s="27" t="s">
         <v>85</v>
       </c>
-      <c r="F25" s="25" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="33"/>
-      <c r="B26" s="33"/>
-      <c r="C26" s="23">
-        <v>21.0</v>
-      </c>
-      <c r="D26" s="24" t="s">
+      <c r="E29" s="27" t="s">
+        <v>65</v>
+      </c>
+      <c r="F29" s="33" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="34"/>
+      <c r="B30" s="31" t="s">
         <v>86</v>
       </c>
-      <c r="E26" s="24" t="s">
+      <c r="C30" s="32">
+        <v>25.0</v>
+      </c>
+      <c r="D30" s="27" t="s">
         <v>87</v>
       </c>
-      <c r="F26" s="25" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="33"/>
-      <c r="B27" s="33"/>
-      <c r="C27" s="23">
-        <v>22.0</v>
-      </c>
-      <c r="D27" s="24" t="s">
+      <c r="E30" s="27" t="s">
         <v>88</v>
       </c>
-      <c r="E27" s="24" t="s">
+      <c r="F30" s="33" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="34"/>
+      <c r="B31" s="34"/>
+      <c r="C31" s="32">
+        <v>26.0</v>
+      </c>
+      <c r="D31" s="27" t="s">
         <v>89</v>
       </c>
-      <c r="F27" s="25" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="33"/>
-      <c r="B28" s="33"/>
-      <c r="C28" s="23">
-        <v>23.0</v>
-      </c>
-      <c r="D28" s="24" t="s">
+      <c r="E31" s="27" t="s">
         <v>90</v>
       </c>
-      <c r="E28" s="24" t="s">
-        <v>76</v>
-      </c>
-      <c r="F28" s="25" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="33"/>
-      <c r="B29" s="33"/>
-      <c r="C29" s="23">
-        <v>24.0</v>
-      </c>
-      <c r="D29" s="24" t="s">
+      <c r="F31" s="33" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="34"/>
+      <c r="B32" s="34"/>
+      <c r="C32" s="32">
+        <v>27.0</v>
+      </c>
+      <c r="D32" s="27" t="s">
         <v>91</v>
       </c>
-      <c r="E29" s="24" t="s">
-        <v>76</v>
-      </c>
-      <c r="F29" s="25" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="33"/>
-      <c r="B30" s="33"/>
-      <c r="C30" s="23">
-        <v>25.0</v>
-      </c>
-      <c r="D30" s="24" t="s">
+      <c r="E32" s="27" t="s">
+        <v>90</v>
+      </c>
+      <c r="F32" s="33" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="34"/>
+      <c r="B33" s="34"/>
+      <c r="C33" s="32">
+        <v>28.0</v>
+      </c>
+      <c r="D33" s="27" t="s">
         <v>92</v>
       </c>
-      <c r="E30" s="24" t="s">
-        <v>60</v>
-      </c>
-      <c r="F30" s="25" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="33"/>
-      <c r="B31" s="33"/>
-      <c r="C31" s="23">
-        <v>26.0</v>
-      </c>
-      <c r="D31" s="24" t="s">
+      <c r="E33" s="27" t="s">
         <v>93</v>
       </c>
-      <c r="E31" s="24" t="s">
-        <v>60</v>
-      </c>
-      <c r="F31" s="25" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="33"/>
-      <c r="B32" s="34"/>
-      <c r="C32" s="23">
-        <v>27.0</v>
-      </c>
-      <c r="D32" s="24" t="s">
+      <c r="F33" s="33" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="34"/>
+      <c r="B34" s="34"/>
+      <c r="C34" s="32">
+        <v>29.0</v>
+      </c>
+      <c r="D34" s="27" t="s">
         <v>94</v>
       </c>
-      <c r="E32" s="24" t="s">
+      <c r="E34" s="27" t="s">
         <v>95</v>
       </c>
-      <c r="F32" s="25" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="33"/>
-      <c r="B33" s="32" t="s">
+      <c r="F34" s="33" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="34"/>
+      <c r="B35" s="34"/>
+      <c r="C35" s="32">
+        <v>30.0</v>
+      </c>
+      <c r="D35" s="27" t="s">
         <v>96</v>
       </c>
-      <c r="C33" s="23">
-        <v>28.0</v>
-      </c>
-      <c r="D33" s="24" t="s">
+      <c r="E35" s="27" t="s">
+        <v>59</v>
+      </c>
+      <c r="F35" s="33" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="34"/>
+      <c r="B36" s="34"/>
+      <c r="C36" s="32">
+        <v>31.0</v>
+      </c>
+      <c r="D36" s="27" t="s">
         <v>97</v>
       </c>
-      <c r="E33" s="24" t="s">
-        <v>83</v>
-      </c>
-      <c r="F33" s="25" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="33"/>
-      <c r="B34" s="33"/>
-      <c r="C34" s="23">
-        <v>29.0</v>
-      </c>
-      <c r="D34" s="24" t="s">
+      <c r="E36" s="27" t="s">
+        <v>59</v>
+      </c>
+      <c r="F36" s="33" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="34"/>
+      <c r="B37" s="34"/>
+      <c r="C37" s="32">
+        <v>32.0</v>
+      </c>
+      <c r="D37" s="27" t="s">
         <v>98</v>
       </c>
-      <c r="E34" s="24" t="s">
+      <c r="E37" s="27" t="s">
         <v>99</v>
       </c>
-      <c r="F34" s="25" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="33"/>
-      <c r="B35" s="33"/>
-      <c r="C35" s="23">
-        <v>30.0</v>
-      </c>
-      <c r="D35" s="24" t="s">
+      <c r="F37" s="33" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="34"/>
+      <c r="B38" s="34"/>
+      <c r="C38" s="32">
+        <v>33.0</v>
+      </c>
+      <c r="D38" s="27" t="s">
         <v>100</v>
       </c>
-      <c r="E35" s="24" t="s">
+      <c r="E38" s="27" t="s">
+        <v>99</v>
+      </c>
+      <c r="F38" s="33" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="34"/>
+      <c r="B39" s="34"/>
+      <c r="C39" s="32">
+        <v>34.0</v>
+      </c>
+      <c r="D39" s="27" t="s">
         <v>101</v>
       </c>
-      <c r="F35" s="25" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="33"/>
-      <c r="B36" s="33"/>
-      <c r="C36" s="23">
-        <v>31.0</v>
-      </c>
-      <c r="D36" s="24" t="s">
+      <c r="E39" s="27" t="s">
+        <v>65</v>
+      </c>
+      <c r="F39" s="33" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="34"/>
+      <c r="B40" s="34"/>
+      <c r="C40" s="32">
+        <v>35.0</v>
+      </c>
+      <c r="D40" s="27" t="s">
         <v>102</v>
       </c>
-      <c r="E36" s="24" t="s">
+      <c r="E40" s="27" t="s">
+        <v>65</v>
+      </c>
+      <c r="F40" s="33" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="34"/>
+      <c r="B41" s="35"/>
+      <c r="C41" s="32">
+        <v>36.0</v>
+      </c>
+      <c r="D41" s="27" t="s">
         <v>103</v>
       </c>
-      <c r="F36" s="25" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="33"/>
-      <c r="B37" s="33"/>
-      <c r="C37" s="23">
-        <v>32.0</v>
-      </c>
-      <c r="D37" s="24" t="s">
+      <c r="E41" s="27" t="s">
+        <v>65</v>
+      </c>
+      <c r="F41" s="33" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="34"/>
+      <c r="B42" s="31" t="s">
         <v>104</v>
       </c>
-      <c r="E37" s="24" t="s">
-        <v>76</v>
-      </c>
-      <c r="F37" s="25" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="33"/>
-      <c r="B38" s="33"/>
-      <c r="C38" s="23">
-        <v>33.0</v>
-      </c>
-      <c r="D38" s="24" t="s">
+      <c r="C42" s="32">
+        <v>37.0</v>
+      </c>
+      <c r="D42" s="27" t="s">
         <v>105</v>
       </c>
-      <c r="E38" s="24" t="s">
+      <c r="E42" s="27" t="s">
         <v>106</v>
       </c>
-      <c r="F38" s="25" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="33"/>
-      <c r="B39" s="33"/>
-      <c r="C39" s="23">
-        <v>34.0</v>
-      </c>
-      <c r="D39" s="24" t="s">
+      <c r="F42" s="33" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="34"/>
+      <c r="B43" s="34"/>
+      <c r="C43" s="32">
+        <v>38.0</v>
+      </c>
+      <c r="D43" s="27" t="s">
         <v>107</v>
       </c>
-      <c r="E39" s="24" t="s">
-        <v>60</v>
-      </c>
-      <c r="F39" s="25" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="33"/>
-      <c r="B40" s="33"/>
-      <c r="C40" s="23">
-        <v>35.0</v>
-      </c>
-      <c r="D40" s="24" t="s">
-        <v>107</v>
-      </c>
-      <c r="E40" s="24" t="s">
-        <v>60</v>
-      </c>
-      <c r="F40" s="25" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="33"/>
-      <c r="B41" s="34"/>
-      <c r="C41" s="23">
-        <v>36.0</v>
-      </c>
-      <c r="D41" s="35" t="s">
+      <c r="E43" s="27" t="s">
         <v>108</v>
       </c>
-      <c r="E41" s="24" t="s">
+      <c r="F43" s="33" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="34"/>
+      <c r="B44" s="34"/>
+      <c r="C44" s="32">
+        <v>39.0</v>
+      </c>
+      <c r="D44" s="27" t="s">
         <v>109</v>
       </c>
-      <c r="F41" s="25" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="13" t="s">
+      <c r="E44" s="27" t="s">
         <v>110</v>
       </c>
-      <c r="B42" s="13"/>
-      <c r="C42" s="13" t="s">
+      <c r="F44" s="33" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="34"/>
+      <c r="B45" s="34"/>
+      <c r="C45" s="32">
+        <v>40.0</v>
+      </c>
+      <c r="D45" s="27" t="s">
         <v>111</v>
       </c>
+      <c r="E45" s="27" t="s">
+        <v>52</v>
+      </c>
+      <c r="F45" s="33" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="34"/>
+      <c r="B46" s="34"/>
+      <c r="C46" s="32">
+        <v>41.0</v>
+      </c>
+      <c r="D46" s="27" t="s">
+        <v>112</v>
+      </c>
+      <c r="E46" s="27" t="s">
+        <v>113</v>
+      </c>
+      <c r="F46" s="33" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="34"/>
+      <c r="B47" s="34"/>
+      <c r="C47" s="32">
+        <v>42.0</v>
+      </c>
+      <c r="D47" s="27" t="s">
+        <v>114</v>
+      </c>
+      <c r="E47" s="27" t="s">
+        <v>59</v>
+      </c>
+      <c r="F47" s="33" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="34"/>
+      <c r="B48" s="34"/>
+      <c r="C48" s="32">
+        <v>43.0</v>
+      </c>
+      <c r="D48" s="27" t="s">
+        <v>115</v>
+      </c>
+      <c r="E48" s="27" t="s">
+        <v>59</v>
+      </c>
+      <c r="F48" s="33" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="34"/>
+      <c r="B49" s="34"/>
+      <c r="C49" s="32">
+        <v>44.0</v>
+      </c>
+      <c r="D49" s="27" t="s">
+        <v>116</v>
+      </c>
+      <c r="E49" s="27" t="s">
+        <v>99</v>
+      </c>
+      <c r="F49" s="33" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="34"/>
+      <c r="B50" s="34"/>
+      <c r="C50" s="32">
+        <v>45.0</v>
+      </c>
+      <c r="D50" s="27" t="s">
+        <v>117</v>
+      </c>
+      <c r="E50" s="27" t="s">
+        <v>118</v>
+      </c>
+      <c r="F50" s="33" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="34"/>
+      <c r="B51" s="34"/>
+      <c r="C51" s="32">
+        <v>46.0</v>
+      </c>
+      <c r="D51" s="27" t="s">
+        <v>119</v>
+      </c>
+      <c r="E51" s="27" t="s">
+        <v>65</v>
+      </c>
+      <c r="F51" s="33" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="34"/>
+      <c r="B52" s="34"/>
+      <c r="C52" s="32">
+        <v>47.0</v>
+      </c>
+      <c r="D52" s="27" t="s">
+        <v>120</v>
+      </c>
+      <c r="E52" s="27" t="s">
+        <v>65</v>
+      </c>
+      <c r="F52" s="33" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="34"/>
+      <c r="B53" s="35"/>
+      <c r="C53" s="32">
+        <v>48.0</v>
+      </c>
+      <c r="D53" s="27" t="s">
+        <v>121</v>
+      </c>
+      <c r="E53" s="27" t="s">
+        <v>65</v>
+      </c>
+      <c r="F53" s="33" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="34"/>
+      <c r="B54" s="36" t="s">
+        <v>122</v>
+      </c>
+      <c r="C54" s="32">
+        <v>49.0</v>
+      </c>
+      <c r="D54" s="26" t="s">
+        <v>123</v>
+      </c>
+      <c r="E54" s="26" t="s">
+        <v>124</v>
+      </c>
+      <c r="F54" s="37" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="34"/>
+      <c r="C55" s="32">
+        <v>50.0</v>
+      </c>
+      <c r="D55" s="26" t="s">
+        <v>125</v>
+      </c>
+      <c r="E55" s="26" t="s">
+        <v>126</v>
+      </c>
+      <c r="F55" s="37" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="34"/>
+      <c r="C56" s="32">
+        <v>51.0</v>
+      </c>
+      <c r="D56" s="26" t="s">
+        <v>127</v>
+      </c>
+      <c r="E56" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="F56" s="37" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="34"/>
+      <c r="C57" s="32">
+        <v>52.0</v>
+      </c>
+      <c r="D57" s="26" t="s">
+        <v>129</v>
+      </c>
+      <c r="E57" s="26" t="s">
+        <v>130</v>
+      </c>
+      <c r="F57" s="37" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="34"/>
+      <c r="C58" s="32">
+        <v>53.0</v>
+      </c>
+      <c r="D58" s="26" t="s">
+        <v>131</v>
+      </c>
+      <c r="E58" s="26" t="s">
+        <v>132</v>
+      </c>
+      <c r="F58" s="37" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="34"/>
+      <c r="C59" s="32">
+        <v>54.0</v>
+      </c>
+      <c r="D59" s="26" t="s">
+        <v>133</v>
+      </c>
+      <c r="E59" s="27" t="s">
+        <v>59</v>
+      </c>
+      <c r="F59" s="37" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="34"/>
+      <c r="C60" s="32">
+        <v>55.0</v>
+      </c>
+      <c r="D60" s="26" t="s">
+        <v>134</v>
+      </c>
+      <c r="E60" s="27" t="s">
+        <v>59</v>
+      </c>
+      <c r="F60" s="37" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="34"/>
+      <c r="C61" s="32">
+        <v>56.0</v>
+      </c>
+      <c r="D61" s="26" t="s">
+        <v>135</v>
+      </c>
+      <c r="E61" s="27" t="s">
+        <v>99</v>
+      </c>
+      <c r="F61" s="37" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="34"/>
+      <c r="C62" s="32">
+        <v>57.0</v>
+      </c>
+      <c r="D62" s="26" t="s">
+        <v>136</v>
+      </c>
+      <c r="E62" s="26" t="s">
+        <v>62</v>
+      </c>
+      <c r="F62" s="37" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="34"/>
+      <c r="C63" s="32">
+        <v>58.0</v>
+      </c>
+      <c r="D63" s="26" t="s">
+        <v>137</v>
+      </c>
+      <c r="E63" s="27" t="s">
+        <v>65</v>
+      </c>
+      <c r="F63" s="37" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="34"/>
+      <c r="C64" s="32">
+        <v>59.0</v>
+      </c>
+      <c r="D64" s="26" t="s">
+        <v>138</v>
+      </c>
+      <c r="E64" s="27" t="s">
+        <v>65</v>
+      </c>
+      <c r="F64" s="37" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="34"/>
+      <c r="C65" s="32">
+        <v>60.0</v>
+      </c>
+      <c r="D65" s="26" t="s">
+        <v>139</v>
+      </c>
+      <c r="E65" s="27" t="s">
+        <v>65</v>
+      </c>
+      <c r="F65" s="37" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="34"/>
+      <c r="B66" s="38" t="s">
+        <v>140</v>
+      </c>
+      <c r="C66" s="32">
+        <v>61.0</v>
+      </c>
+      <c r="D66" s="26" t="s">
+        <v>141</v>
+      </c>
+      <c r="E66" s="26" t="s">
+        <v>142</v>
+      </c>
+      <c r="F66" s="37" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="34"/>
+      <c r="B67" s="34"/>
+      <c r="C67" s="32">
+        <v>63.0</v>
+      </c>
+      <c r="D67" s="26" t="s">
+        <v>143</v>
+      </c>
+      <c r="E67" s="26" t="s">
+        <v>144</v>
+      </c>
+      <c r="F67" s="37" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="34"/>
+      <c r="B68" s="34"/>
+      <c r="C68" s="32">
+        <v>65.0</v>
+      </c>
+      <c r="D68" s="26" t="s">
+        <v>145</v>
+      </c>
+      <c r="E68" s="26" t="s">
+        <v>146</v>
+      </c>
+      <c r="F68" s="37" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="34"/>
+      <c r="B69" s="34"/>
+      <c r="C69" s="32">
+        <v>66.0</v>
+      </c>
+      <c r="D69" s="26" t="s">
+        <v>147</v>
+      </c>
+      <c r="E69" s="27" t="s">
+        <v>59</v>
+      </c>
+      <c r="F69" s="37" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="34"/>
+      <c r="B70" s="34"/>
+      <c r="C70" s="32">
+        <v>68.0</v>
+      </c>
+      <c r="D70" s="26" t="s">
+        <v>148</v>
+      </c>
+      <c r="E70" s="27" t="s">
+        <v>99</v>
+      </c>
+      <c r="F70" s="37" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="34"/>
+      <c r="B71" s="35"/>
+      <c r="C71" s="32">
+        <v>70.0</v>
+      </c>
+      <c r="D71" s="26" t="s">
+        <v>149</v>
+      </c>
+      <c r="E71" s="27" t="s">
+        <v>65</v>
+      </c>
+      <c r="F71" s="37" t="b">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="10">
-    <mergeCell ref="B15:B23"/>
-    <mergeCell ref="B24:B32"/>
+  <mergeCells count="11">
+    <mergeCell ref="B30:B41"/>
+    <mergeCell ref="B42:B53"/>
+    <mergeCell ref="B54:B65"/>
+    <mergeCell ref="B66:B71"/>
+    <mergeCell ref="A6:A71"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A3:F3"/>
     <mergeCell ref="A4:F4"/>
-    <mergeCell ref="C42:F42"/>
-    <mergeCell ref="B6:B14"/>
-    <mergeCell ref="B33:B41"/>
-    <mergeCell ref="A6:A41"/>
+    <mergeCell ref="B6:B17"/>
+    <mergeCell ref="B18:B29"/>
   </mergeCells>
   <printOptions gridLines="1" horizontalCentered="1"/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>

</xml_diff>